<commit_message>
Update September 2026: new participant numbering (starting at 28), new retrieval trials (only order and distance questions, only distances 2-5 covered), retrieval trials now include reflection period and practice trials include backgroundinformation about the example sequence
</commit_message>
<xml_diff>
--- a/sequences/main_trials_prc.xlsx
+++ b/sequences/main_trials_prc.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sync_folder\TSRlearn-task\sequences\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sync_folder\TSRlearn_BIE\sequences\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -68,9 +68,6 @@
     <t>y</t>
   </si>
   <si>
-    <t>stimuli/practice_images/anchor.jpg</t>
-  </si>
-  <si>
     <t>stimuli/practice_images/cow.jpg</t>
   </si>
   <si>
@@ -111,6 +108,9 @@
   </si>
   <si>
     <t>stimuli/practice_images/bird.jpg</t>
+  </si>
+  <si>
+    <t>stimuli/practice_images/broom.jpg</t>
   </si>
 </sst>
 </file>
@@ -463,16 +463,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>16</v>
-      </c>
-      <c r="D2" t="s">
-        <v>17</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -489,16 +489,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
       </c>
       <c r="E3" t="s">
         <v>9</v>
@@ -515,16 +515,16 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -541,16 +541,16 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -567,16 +567,16 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
         <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -593,16 +593,16 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>

</xml_diff>